<commit_message>
update .gitignore , create the lab 4 work , complete heap sort analysis , update quick sort
</commit_message>
<xml_diff>
--- a/lab/quickSortComplexityAnalysis.xlsx
+++ b/lab/quickSortComplexityAnalysis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d563af19fdf9b553/Documents/GitHub/Design-And-Analysis-of-Algorithm/lab/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2EBC8B34-6C28-4D8B-870C-25D8F3CDA44F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{2EBC8B34-6C28-4D8B-870C-25D8F3CDA44F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10A291C6-25FF-4187-BDBA-1AD1D95F1552}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A9386D12-26EA-4D90-BE84-F38A622FA1EF}"/>
   </bookViews>
@@ -172,7 +172,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-IN"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2866,15 +2866,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>350520</xdr:colOff>
-      <xdr:row>73</xdr:row>
-      <xdr:rowOff>175260</xdr:rowOff>
+      <xdr:colOff>259080</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>365760</xdr:colOff>
-      <xdr:row>97</xdr:row>
-      <xdr:rowOff>106680</xdr:rowOff>
+      <xdr:colOff>274320</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>